<commit_message>
chore: actualizar plantilla de paleta
</commit_message>
<xml_diff>
--- a/chancado/analytica/Report/Lote-Export-Base.xlsx
+++ b/chancado/analytica/Report/Lote-Export-Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\chancado\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E05B10-5618-44FC-97A3-CA853A7DD48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E968EA4C-3610-4A95-AF36-20B6654B8581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;S/ &quot;* #,##0.00_-;&quot;-S/ &quot;* #,##0.00_-;_-&quot;S/ &quot;* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -143,6 +143,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -239,9 +245,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -259,6 +262,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="24">
@@ -614,17 +620,17 @@
       <c r="AY1" s="3"/>
     </row>
     <row r="2" spans="1:51" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
       <c r="J2" s="2"/>
       <c r="K2" s="4"/>
       <c r="L2" s="3"/>
@@ -669,17 +675,17 @@
       <c r="AY2" s="3"/>
     </row>
     <row r="3" spans="1:51" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
       <c r="J3" s="1"/>
       <c r="K3" s="5"/>
       <c r="L3" s="3"/>
@@ -794,14 +800,14 @@
       <c r="B6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="10"/>
+      <c r="C6" s="16"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="11"/>
+      <c r="H6" s="10"/>
       <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:51" ht="18" x14ac:dyDescent="0.3">
@@ -818,41 +824,41 @@
       <c r="K7" s="6"/>
     </row>
     <row r="8" spans="1:51" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="12" t="s">
+      <c r="K8" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:51" s="13" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:51" s="12" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:51" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
chore: actualizar plantilla de exportacion de excel
</commit_message>
<xml_diff>
--- a/chancado/analytica/Report/Lote-Export-Base.xlsx
+++ b/chancado/analytica/Report/Lote-Export-Base.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\chancado\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E968EA4C-3610-4A95-AF36-20B6654B8581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{932B5DFD-B31E-42BE-BBF1-30EA09EECC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;S/ &quot;* #,##0.00_-;&quot;-S/ &quot;* #,##0.00_-;_-&quot;S/ &quot;* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -147,12 +147,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -263,7 +257,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="22" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -562,7 +556,7 @@
     <col min="7" max="7" width="25.77734375" customWidth="1"/>
     <col min="8" max="8" width="28.5546875" customWidth="1"/>
     <col min="9" max="9" width="24.77734375" customWidth="1"/>
-    <col min="10" max="10" width="14.88671875" customWidth="1"/>
+    <col min="10" max="10" width="23.6640625" customWidth="1"/>
     <col min="11" max="11" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
feat: actualizar nombre de columna obs balanza a solo observacion en excel chancado
</commit_message>
<xml_diff>
--- a/chancado/analytica/Report/Lote-Export-Base.xlsx
+++ b/chancado/analytica/Report/Lote-Export-Base.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\chancado\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07324D3-CB26-4942-9009-A75BC81F7534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C4ED79-AD3E-4035-A865-24991389F6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,9 +57,6 @@
     <t>PLACA CARRETA</t>
   </si>
   <si>
-    <t>OBS. BALANZA</t>
-  </si>
-  <si>
     <t>CANCHA</t>
   </si>
   <si>
@@ -76,6 +73,9 @@
   </si>
   <si>
     <t>ESTADO PESAJE</t>
+  </si>
+  <si>
+    <t>OBSERVACION</t>
   </si>
 </sst>
 </file>
@@ -841,28 +841,28 @@
         <v>9</v>
       </c>
       <c r="G8" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="I8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="J8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="K8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="11" t="s">
-        <v>14</v>
-      </c>
       <c r="L8" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:51" s="12" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:51" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: actualizar plantilla de chancado
</commit_message>
<xml_diff>
--- a/chancado/analytica/Report/Lote-Export-Base.xlsx
+++ b/chancado/analytica/Report/Lote-Export-Base.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\projects\minersoft-projects\minersoft\acopio-project-configuration\chancado\analytica\Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C4ED79-AD3E-4035-A865-24991389F6E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4538292B-3A6F-4ABA-94ED-E6D5E6D2B614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,7 +75,7 @@
     <t>ESTADO PESAJE</t>
   </si>
   <si>
-    <t>OBSERVACION</t>
+    <t>OBSERVACIÓN BALANZA</t>
   </si>
 </sst>
 </file>

</xml_diff>